<commit_message>
feat: mostra as matrizes originais ao lado do resultado
Cada aba de resultado ganha, na linha 12, blocos lado a lado:
originais | resultado | probabilidades.
- misturar: originais A e B
- reconstruir: exemplo original
- gerar: exemplo de treino mais parecido
O terminal mostra as mesmas matrizes lado a lado.
</commit_message>
<xml_diff>
--- a/exemplos/misturas_0_8.xlsx
+++ b/exemplos/misturas_0_8.xlsx
@@ -492,7 +492,7 @@
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t>A12:F19: probabilidades antes do limiar, em escala de cores fixa de 0 a 1.</t>
+          <t>Linha 12, lado a lado: matrizes originais, resultado e probabilidades antes do limiar.</t>
         </is>
       </c>
     </row>
@@ -529,174 +529,669 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="0" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Original 0 (A)</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Original 8 (B)</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>Resultado</t>
+        </is>
+      </c>
+      <c r="V11" s="5" t="inlineStr">
         <is>
           <t>Probabilidades</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4">
+      <c r="A12" s="1">
+        <v>0</v>
+      </c>
+      <c r="B12" s="1">
+        <v>0</v>
+      </c>
+      <c r="C12" s="1">
+        <v>0</v>
+      </c>
+      <c r="D12" s="1">
+        <v>0</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0</v>
+      </c>
+      <c r="F12" s="1">
+        <v>0</v>
+      </c>
+      <c r="H12" s="1">
+        <v>0</v>
+      </c>
+      <c r="I12" s="1">
+        <v>0</v>
+      </c>
+      <c r="J12" s="1">
+        <v>0</v>
+      </c>
+      <c r="K12" s="1">
+        <v>0</v>
+      </c>
+      <c r="L12" s="1">
+        <v>0</v>
+      </c>
+      <c r="M12" s="1">
+        <v>0</v>
+      </c>
+      <c r="O12" s="1">
+        <f>A1</f>
+        <v>0</v>
+      </c>
+      <c r="P12" s="1">
+        <f>B1</f>
+        <v>0</v>
+      </c>
+      <c r="Q12" s="1">
+        <f>C1</f>
+        <v>0</v>
+      </c>
+      <c r="R12" s="1">
+        <f>D1</f>
+        <v>0</v>
+      </c>
+      <c r="S12" s="1">
+        <f>E1</f>
+        <v>0</v>
+      </c>
+      <c r="T12" s="1">
+        <f>F1</f>
+        <v>0</v>
+      </c>
+      <c r="V12" s="4">
         <v>4.7870413484011178e-05</v>
       </c>
-      <c r="B12" s="4">
+      <c r="W12" s="4">
         <v>3.8204514190829057e-05</v>
       </c>
-      <c r="C12" s="4">
+      <c r="X12" s="4">
         <v>5.0551732708527279e-05</v>
       </c>
-      <c r="D12" s="4">
+      <c r="Y12" s="4">
         <v>3.6520379375831005e-05</v>
       </c>
-      <c r="E12" s="4">
+      <c r="Z12" s="4">
         <v>9.0820784399591261e-05</v>
       </c>
-      <c r="F12" s="4">
+      <c r="AA12" s="4">
         <v>3.9987158430999814e-05</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4">
+      <c r="A13" s="1">
+        <v>0</v>
+      </c>
+      <c r="B13" s="1">
+        <v>0</v>
+      </c>
+      <c r="C13" s="1">
+        <v>1</v>
+      </c>
+      <c r="D13" s="1">
+        <v>1</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0</v>
+      </c>
+      <c r="H13" s="1">
+        <v>0</v>
+      </c>
+      <c r="I13" s="1">
+        <v>0</v>
+      </c>
+      <c r="J13" s="1">
+        <v>1</v>
+      </c>
+      <c r="K13" s="1">
+        <v>1</v>
+      </c>
+      <c r="L13" s="1">
+        <v>0</v>
+      </c>
+      <c r="M13" s="1">
+        <v>0</v>
+      </c>
+      <c r="O13" s="1">
+        <f>A2</f>
+        <v>0</v>
+      </c>
+      <c r="P13" s="1">
+        <f>B2</f>
+        <v>0</v>
+      </c>
+      <c r="Q13" s="1">
+        <f>C2</f>
+        <v>1</v>
+      </c>
+      <c r="R13" s="1">
+        <f>D2</f>
+        <v>1</v>
+      </c>
+      <c r="S13" s="1">
+        <f>E2</f>
+        <v>0</v>
+      </c>
+      <c r="T13" s="1">
+        <f>F2</f>
+        <v>0</v>
+      </c>
+      <c r="V13" s="4">
         <v>2.5410513526453375e-05</v>
       </c>
-      <c r="B13" s="4">
+      <c r="W13" s="4">
         <v>5.399435370840253e-06</v>
       </c>
-      <c r="C13" s="4">
+      <c r="X13" s="4">
         <v>0.9999954178675895</v>
       </c>
-      <c r="D13" s="4">
+      <c r="Y13" s="4">
         <v>0.99986113954126254</v>
       </c>
-      <c r="E13" s="4">
+      <c r="Z13" s="4">
         <v>1.9647931669477483e-06</v>
       </c>
-      <c r="F13" s="4">
+      <c r="AA13" s="4">
         <v>3.9083110521726453e-05</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4">
+      <c r="A14" s="1">
+        <v>0</v>
+      </c>
+      <c r="B14" s="1">
+        <v>1</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1">
+        <v>1</v>
+      </c>
+      <c r="F14" s="1">
+        <v>0</v>
+      </c>
+      <c r="H14" s="1">
+        <v>0</v>
+      </c>
+      <c r="I14" s="1">
+        <v>1</v>
+      </c>
+      <c r="J14" s="1">
+        <v>0</v>
+      </c>
+      <c r="K14" s="1">
+        <v>0</v>
+      </c>
+      <c r="L14" s="1">
+        <v>1</v>
+      </c>
+      <c r="M14" s="1">
+        <v>0</v>
+      </c>
+      <c r="O14" s="1">
+        <f>A3</f>
+        <v>0</v>
+      </c>
+      <c r="P14" s="1">
+        <f>B3</f>
+        <v>1</v>
+      </c>
+      <c r="Q14" s="1">
+        <f>C3</f>
+        <v>0</v>
+      </c>
+      <c r="R14" s="1">
+        <f>D3</f>
+        <v>0</v>
+      </c>
+      <c r="S14" s="1">
+        <f>E3</f>
+        <v>1</v>
+      </c>
+      <c r="T14" s="1">
+        <f>F3</f>
+        <v>0</v>
+      </c>
+      <c r="V14" s="4">
         <v>3.4757283671835729e-05</v>
       </c>
-      <c r="B14" s="4">
+      <c r="W14" s="4">
         <v>0.99999999308911036</v>
       </c>
-      <c r="C14" s="4">
+      <c r="X14" s="4">
         <v>2.8248627735024196e-07</v>
       </c>
-      <c r="D14" s="4">
+      <c r="Y14" s="4">
         <v>1.6181671245320351e-09</v>
       </c>
-      <c r="E14" s="4">
+      <c r="Z14" s="4">
         <v>0.9999999977543641</v>
       </c>
-      <c r="F14" s="4">
+      <c r="AA14" s="4">
         <v>2.1602196875778644e-05</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4">
+      <c r="A15" s="1">
+        <v>0</v>
+      </c>
+      <c r="B15" s="1">
+        <v>1</v>
+      </c>
+      <c r="C15" s="1">
+        <v>0</v>
+      </c>
+      <c r="D15" s="1">
+        <v>0</v>
+      </c>
+      <c r="E15" s="1">
+        <v>1</v>
+      </c>
+      <c r="F15" s="1">
+        <v>0</v>
+      </c>
+      <c r="H15" s="1">
+        <v>0</v>
+      </c>
+      <c r="I15" s="1">
+        <v>0</v>
+      </c>
+      <c r="J15" s="1">
+        <v>1</v>
+      </c>
+      <c r="K15" s="1">
+        <v>1</v>
+      </c>
+      <c r="L15" s="1">
+        <v>0</v>
+      </c>
+      <c r="M15" s="1">
+        <v>0</v>
+      </c>
+      <c r="O15" s="1">
+        <f>A4</f>
+        <v>0</v>
+      </c>
+      <c r="P15" s="1">
+        <f>B4</f>
+        <v>1</v>
+      </c>
+      <c r="Q15" s="1">
+        <f>C4</f>
+        <v>0</v>
+      </c>
+      <c r="R15" s="1">
+        <f>D4</f>
+        <v>0</v>
+      </c>
+      <c r="S15" s="1">
+        <f>E4</f>
+        <v>1</v>
+      </c>
+      <c r="T15" s="1">
+        <f>F4</f>
+        <v>0</v>
+      </c>
+      <c r="V15" s="4">
         <v>2.5168466652210865e-05</v>
       </c>
-      <c r="B15" s="4">
+      <c r="W15" s="4">
         <v>0.99947099645995652</v>
       </c>
-      <c r="C15" s="4">
+      <c r="X15" s="4">
         <v>0.00062017934831232386</v>
       </c>
-      <c r="D15" s="4">
+      <c r="Y15" s="4">
         <v>0.00049684944991581267</v>
       </c>
-      <c r="E15" s="4">
+      <c r="Z15" s="4">
         <v>0.99995966237588652</v>
       </c>
-      <c r="F15" s="4">
+      <c r="AA15" s="4">
         <v>3.1671099700741616e-05</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4">
+      <c r="A16" s="1">
+        <v>0</v>
+      </c>
+      <c r="B16" s="1">
+        <v>1</v>
+      </c>
+      <c r="C16" s="1">
+        <v>0</v>
+      </c>
+      <c r="D16" s="1">
+        <v>0</v>
+      </c>
+      <c r="E16" s="1">
+        <v>1</v>
+      </c>
+      <c r="F16" s="1">
+        <v>0</v>
+      </c>
+      <c r="H16" s="1">
+        <v>0</v>
+      </c>
+      <c r="I16" s="1">
+        <v>1</v>
+      </c>
+      <c r="J16" s="1">
+        <v>0</v>
+      </c>
+      <c r="K16" s="1">
+        <v>0</v>
+      </c>
+      <c r="L16" s="1">
+        <v>1</v>
+      </c>
+      <c r="M16" s="1">
+        <v>0</v>
+      </c>
+      <c r="O16" s="1">
+        <f>A5</f>
+        <v>0</v>
+      </c>
+      <c r="P16" s="1">
+        <f>B5</f>
+        <v>1</v>
+      </c>
+      <c r="Q16" s="1">
+        <f>C5</f>
+        <v>0</v>
+      </c>
+      <c r="R16" s="1">
+        <f>D5</f>
+        <v>0</v>
+      </c>
+      <c r="S16" s="1">
+        <f>E5</f>
+        <v>1</v>
+      </c>
+      <c r="T16" s="1">
+        <f>F5</f>
+        <v>0</v>
+      </c>
+      <c r="V16" s="4">
         <v>3.8050390969611303e-05</v>
       </c>
-      <c r="B16" s="4">
+      <c r="W16" s="4">
         <v>0.9999858601149707</v>
       </c>
-      <c r="C16" s="4">
+      <c r="X16" s="4">
         <v>0.00043489996120470295</v>
       </c>
-      <c r="D16" s="4">
+      <c r="Y16" s="4">
         <v>0.00020044667640124153</v>
       </c>
-      <c r="E16" s="4">
+      <c r="Z16" s="4">
         <v>0.99977014008049925</v>
       </c>
-      <c r="F16" s="4">
+      <c r="AA16" s="4">
         <v>4.4179951725916085e-05</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4">
+      <c r="A17" s="1">
+        <v>0</v>
+      </c>
+      <c r="B17" s="1">
+        <v>1</v>
+      </c>
+      <c r="C17" s="1">
+        <v>0</v>
+      </c>
+      <c r="D17" s="1">
+        <v>0</v>
+      </c>
+      <c r="E17" s="1">
+        <v>1</v>
+      </c>
+      <c r="F17" s="1">
+        <v>0</v>
+      </c>
+      <c r="H17" s="1">
+        <v>0</v>
+      </c>
+      <c r="I17" s="1">
+        <v>1</v>
+      </c>
+      <c r="J17" s="1">
+        <v>0</v>
+      </c>
+      <c r="K17" s="1">
+        <v>0</v>
+      </c>
+      <c r="L17" s="1">
+        <v>1</v>
+      </c>
+      <c r="M17" s="1">
+        <v>0</v>
+      </c>
+      <c r="O17" s="1">
+        <f>A6</f>
+        <v>0</v>
+      </c>
+      <c r="P17" s="1">
+        <f>B6</f>
+        <v>1</v>
+      </c>
+      <c r="Q17" s="1">
+        <f>C6</f>
+        <v>0</v>
+      </c>
+      <c r="R17" s="1">
+        <f>D6</f>
+        <v>0</v>
+      </c>
+      <c r="S17" s="1">
+        <f>E6</f>
+        <v>1</v>
+      </c>
+      <c r="T17" s="1">
+        <f>F6</f>
+        <v>0</v>
+      </c>
+      <c r="V17" s="4">
         <v>2.2936272100302958e-05</v>
       </c>
-      <c r="B17" s="4">
+      <c r="W17" s="4">
         <v>0.99990337592811518</v>
       </c>
-      <c r="C17" s="4">
+      <c r="X17" s="4">
         <v>3.7759381938189797e-05</v>
       </c>
-      <c r="D17" s="4">
+      <c r="Y17" s="4">
         <v>1.2586903305225215e-07</v>
       </c>
-      <c r="E17" s="4">
+      <c r="Z17" s="4">
         <v>0.99999975522557727</v>
       </c>
-      <c r="F17" s="4">
+      <c r="AA17" s="4">
         <v>5.2083207754666432e-05</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4">
+      <c r="A18" s="1">
+        <v>0</v>
+      </c>
+      <c r="B18" s="1">
+        <v>0</v>
+      </c>
+      <c r="C18" s="1">
+        <v>1</v>
+      </c>
+      <c r="D18" s="1">
+        <v>1</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0</v>
+      </c>
+      <c r="F18" s="1">
+        <v>0</v>
+      </c>
+      <c r="H18" s="1">
+        <v>0</v>
+      </c>
+      <c r="I18" s="1">
+        <v>0</v>
+      </c>
+      <c r="J18" s="1">
+        <v>1</v>
+      </c>
+      <c r="K18" s="1">
+        <v>1</v>
+      </c>
+      <c r="L18" s="1">
+        <v>0</v>
+      </c>
+      <c r="M18" s="1">
+        <v>0</v>
+      </c>
+      <c r="O18" s="1">
+        <f>A7</f>
+        <v>0</v>
+      </c>
+      <c r="P18" s="1">
+        <f>B7</f>
+        <v>0</v>
+      </c>
+      <c r="Q18" s="1">
+        <f>C7</f>
+        <v>1</v>
+      </c>
+      <c r="R18" s="1">
+        <f>D7</f>
+        <v>1</v>
+      </c>
+      <c r="S18" s="1">
+        <f>E7</f>
+        <v>0</v>
+      </c>
+      <c r="T18" s="1">
+        <f>F7</f>
+        <v>0</v>
+      </c>
+      <c r="V18" s="4">
         <v>3.2899034852019231e-05</v>
       </c>
-      <c r="B18" s="4">
+      <c r="W18" s="4">
         <v>4.0230436454734512e-08</v>
       </c>
-      <c r="C18" s="4">
+      <c r="X18" s="4">
         <v>0.99987606160865672</v>
       </c>
-      <c r="D18" s="4">
+      <c r="Y18" s="4">
         <v>0.99985616425509827</v>
       </c>
-      <c r="E18" s="4">
+      <c r="Z18" s="4">
         <v>3.6289367009589144e-06</v>
       </c>
-      <c r="F18" s="4">
+      <c r="AA18" s="4">
         <v>3.3530699729301213e-05</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4">
+      <c r="A19" s="1">
+        <v>0</v>
+      </c>
+      <c r="B19" s="1">
+        <v>0</v>
+      </c>
+      <c r="C19" s="1">
+        <v>0</v>
+      </c>
+      <c r="D19" s="1">
+        <v>0</v>
+      </c>
+      <c r="E19" s="1">
+        <v>0</v>
+      </c>
+      <c r="F19" s="1">
+        <v>0</v>
+      </c>
+      <c r="H19" s="1">
+        <v>0</v>
+      </c>
+      <c r="I19" s="1">
+        <v>0</v>
+      </c>
+      <c r="J19" s="1">
+        <v>0</v>
+      </c>
+      <c r="K19" s="1">
+        <v>0</v>
+      </c>
+      <c r="L19" s="1">
+        <v>0</v>
+      </c>
+      <c r="M19" s="1">
+        <v>0</v>
+      </c>
+      <c r="O19" s="1">
+        <f>A8</f>
+        <v>0</v>
+      </c>
+      <c r="P19" s="1">
+        <f>B8</f>
+        <v>0</v>
+      </c>
+      <c r="Q19" s="1">
+        <f>C8</f>
+        <v>0</v>
+      </c>
+      <c r="R19" s="1">
+        <f>D8</f>
+        <v>0</v>
+      </c>
+      <c r="S19" s="1">
+        <f>E8</f>
+        <v>0</v>
+      </c>
+      <c r="T19" s="1">
+        <f>F8</f>
+        <v>0</v>
+      </c>
+      <c r="V19" s="4">
         <v>3.9289112676993288e-05</v>
       </c>
-      <c r="B19" s="4">
+      <c r="W19" s="4">
         <v>4.7633284506401324e-05</v>
       </c>
-      <c r="C19" s="4">
+      <c r="X19" s="4">
         <v>6.1997765261549167e-05</v>
       </c>
-      <c r="D19" s="4">
+      <c r="Y19" s="4">
         <v>3.5137561073643518e-05</v>
       </c>
-      <c r="E19" s="4">
+      <c r="Z19" s="4">
         <v>5.470528472847099e-05</v>
       </c>
-      <c r="F19" s="4">
+      <c r="AA19" s="4">
         <v>3.7266933298921631e-05</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:F8 H1:BC1">
+  <conditionalFormatting sqref="A1:F8 H1:BC1 A12:F19 H12:M19 O12:T19">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThanOrEqual">
       <formula>0.5</formula>
     </cfRule>
@@ -704,7 +1199,7 @@
       <formula>0.5</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A12:F19">
+  <conditionalFormatting sqref="V12:AA19">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -1086,7 +1581,7 @@
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t>A12:F19: probabilidades antes do limiar, em escala de cores fixa de 0 a 1.</t>
+          <t>Linha 12, lado a lado: matrizes originais, resultado e probabilidades antes do limiar.</t>
         </is>
       </c>
     </row>
@@ -1123,174 +1618,669 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="0" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Original 0 (A)</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Original 8 (B)</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>Resultado</t>
+        </is>
+      </c>
+      <c r="V11" s="5" t="inlineStr">
         <is>
           <t>Probabilidades</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4">
+      <c r="A12" s="1">
+        <v>0</v>
+      </c>
+      <c r="B12" s="1">
+        <v>0</v>
+      </c>
+      <c r="C12" s="1">
+        <v>0</v>
+      </c>
+      <c r="D12" s="1">
+        <v>0</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0</v>
+      </c>
+      <c r="F12" s="1">
+        <v>0</v>
+      </c>
+      <c r="H12" s="1">
+        <v>0</v>
+      </c>
+      <c r="I12" s="1">
+        <v>0</v>
+      </c>
+      <c r="J12" s="1">
+        <v>0</v>
+      </c>
+      <c r="K12" s="1">
+        <v>0</v>
+      </c>
+      <c r="L12" s="1">
+        <v>0</v>
+      </c>
+      <c r="M12" s="1">
+        <v>0</v>
+      </c>
+      <c r="O12" s="1">
+        <f>A1</f>
+        <v>0</v>
+      </c>
+      <c r="P12" s="1">
+        <f>B1</f>
+        <v>0</v>
+      </c>
+      <c r="Q12" s="1">
+        <f>C1</f>
+        <v>0</v>
+      </c>
+      <c r="R12" s="1">
+        <f>D1</f>
+        <v>0</v>
+      </c>
+      <c r="S12" s="1">
+        <f>E1</f>
+        <v>0</v>
+      </c>
+      <c r="T12" s="1">
+        <f>F1</f>
+        <v>0</v>
+      </c>
+      <c r="V12" s="4">
         <v>2.7117324631963118e-05</v>
       </c>
-      <c r="B12" s="4">
+      <c r="W12" s="4">
         <v>2.05209527348743e-05</v>
       </c>
-      <c r="C12" s="4">
+      <c r="X12" s="4">
         <v>2.7930250158766605e-05</v>
       </c>
-      <c r="D12" s="4">
+      <c r="Y12" s="4">
         <v>1.8933444759184925e-05</v>
       </c>
-      <c r="E12" s="4">
+      <c r="Z12" s="4">
         <v>4.6944115009050524e-05</v>
       </c>
-      <c r="F12" s="4">
+      <c r="AA12" s="4">
         <v>2.1859818816034977e-05</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4">
+      <c r="A13" s="1">
+        <v>0</v>
+      </c>
+      <c r="B13" s="1">
+        <v>0</v>
+      </c>
+      <c r="C13" s="1">
+        <v>1</v>
+      </c>
+      <c r="D13" s="1">
+        <v>1</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0</v>
+      </c>
+      <c r="H13" s="1">
+        <v>0</v>
+      </c>
+      <c r="I13" s="1">
+        <v>0</v>
+      </c>
+      <c r="J13" s="1">
+        <v>1</v>
+      </c>
+      <c r="K13" s="1">
+        <v>1</v>
+      </c>
+      <c r="L13" s="1">
+        <v>0</v>
+      </c>
+      <c r="M13" s="1">
+        <v>0</v>
+      </c>
+      <c r="O13" s="1">
+        <f>A2</f>
+        <v>0</v>
+      </c>
+      <c r="P13" s="1">
+        <f>B2</f>
+        <v>0</v>
+      </c>
+      <c r="Q13" s="1">
+        <f>C2</f>
+        <v>1</v>
+      </c>
+      <c r="R13" s="1">
+        <f>D2</f>
+        <v>1</v>
+      </c>
+      <c r="S13" s="1">
+        <f>E2</f>
+        <v>0</v>
+      </c>
+      <c r="T13" s="1">
+        <f>F2</f>
+        <v>0</v>
+      </c>
+      <c r="V13" s="4">
         <v>1.2611112940809079e-05</v>
       </c>
-      <c r="B13" s="4">
+      <c r="W13" s="4">
         <v>5.8822571047085361e-06</v>
       </c>
-      <c r="C13" s="4">
+      <c r="X13" s="4">
         <v>0.99999852205856488</v>
       </c>
-      <c r="D13" s="4">
+      <c r="Y13" s="4">
         <v>0.99995581298202996</v>
       </c>
-      <c r="E13" s="4">
+      <c r="Z13" s="4">
         <v>2.4301265727580247e-06</v>
       </c>
-      <c r="F13" s="4">
+      <c r="AA13" s="4">
         <v>2.1522074214100971e-05</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4">
+      <c r="A14" s="1">
+        <v>0</v>
+      </c>
+      <c r="B14" s="1">
+        <v>1</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1">
+        <v>1</v>
+      </c>
+      <c r="F14" s="1">
+        <v>0</v>
+      </c>
+      <c r="H14" s="1">
+        <v>0</v>
+      </c>
+      <c r="I14" s="1">
+        <v>1</v>
+      </c>
+      <c r="J14" s="1">
+        <v>0</v>
+      </c>
+      <c r="K14" s="1">
+        <v>0</v>
+      </c>
+      <c r="L14" s="1">
+        <v>1</v>
+      </c>
+      <c r="M14" s="1">
+        <v>0</v>
+      </c>
+      <c r="O14" s="1">
+        <f>A3</f>
+        <v>0</v>
+      </c>
+      <c r="P14" s="1">
+        <f>B3</f>
+        <v>1</v>
+      </c>
+      <c r="Q14" s="1">
+        <f>C3</f>
+        <v>0</v>
+      </c>
+      <c r="R14" s="1">
+        <f>D3</f>
+        <v>0</v>
+      </c>
+      <c r="S14" s="1">
+        <f>E3</f>
+        <v>1</v>
+      </c>
+      <c r="T14" s="1">
+        <f>F3</f>
+        <v>0</v>
+      </c>
+      <c r="V14" s="4">
         <v>1.8735354854297269e-05</v>
       </c>
-      <c r="B14" s="4">
+      <c r="W14" s="4">
         <v>0.999999990659037</v>
       </c>
-      <c r="C14" s="4">
+      <c r="X14" s="4">
         <v>1.7584367871202624e-07</v>
       </c>
-      <c r="D14" s="4">
+      <c r="Y14" s="4">
         <v>2.2510974418969141e-09</v>
       </c>
-      <c r="E14" s="4">
+      <c r="Z14" s="4">
         <v>0.99999999510295923</v>
       </c>
-      <c r="F14" s="4">
+      <c r="AA14" s="4">
         <v>1.0425115689357478e-05</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4">
+      <c r="A15" s="1">
+        <v>0</v>
+      </c>
+      <c r="B15" s="1">
+        <v>1</v>
+      </c>
+      <c r="C15" s="1">
+        <v>0</v>
+      </c>
+      <c r="D15" s="1">
+        <v>0</v>
+      </c>
+      <c r="E15" s="1">
+        <v>1</v>
+      </c>
+      <c r="F15" s="1">
+        <v>0</v>
+      </c>
+      <c r="H15" s="1">
+        <v>0</v>
+      </c>
+      <c r="I15" s="1">
+        <v>0</v>
+      </c>
+      <c r="J15" s="1">
+        <v>1</v>
+      </c>
+      <c r="K15" s="1">
+        <v>1</v>
+      </c>
+      <c r="L15" s="1">
+        <v>0</v>
+      </c>
+      <c r="M15" s="1">
+        <v>0</v>
+      </c>
+      <c r="O15" s="1">
+        <f>A4</f>
+        <v>0</v>
+      </c>
+      <c r="P15" s="1">
+        <f>B4</f>
+        <v>1</v>
+      </c>
+      <c r="Q15" s="1">
+        <f>C4</f>
+        <v>0</v>
+      </c>
+      <c r="R15" s="1">
+        <f>D4</f>
+        <v>0</v>
+      </c>
+      <c r="S15" s="1">
+        <f>E4</f>
+        <v>1</v>
+      </c>
+      <c r="T15" s="1">
+        <f>F4</f>
+        <v>0</v>
+      </c>
+      <c r="V15" s="4">
         <v>1.1765775983190302e-05</v>
       </c>
-      <c r="B15" s="4">
+      <c r="W15" s="4">
         <v>0.99789657754024053</v>
       </c>
-      <c r="C15" s="4">
+      <c r="X15" s="4">
         <v>0.0029244189843500548</v>
       </c>
-      <c r="D15" s="4">
+      <c r="Y15" s="4">
         <v>0.0018705764588665276</v>
       </c>
-      <c r="E15" s="4">
+      <c r="Z15" s="4">
         <v>0.99944202987438258</v>
       </c>
-      <c r="F15" s="4">
+      <c r="AA15" s="4">
         <v>1.5279285694111781e-05</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4">
+      <c r="A16" s="1">
+        <v>0</v>
+      </c>
+      <c r="B16" s="1">
+        <v>1</v>
+      </c>
+      <c r="C16" s="1">
+        <v>0</v>
+      </c>
+      <c r="D16" s="1">
+        <v>0</v>
+      </c>
+      <c r="E16" s="1">
+        <v>1</v>
+      </c>
+      <c r="F16" s="1">
+        <v>0</v>
+      </c>
+      <c r="H16" s="1">
+        <v>0</v>
+      </c>
+      <c r="I16" s="1">
+        <v>1</v>
+      </c>
+      <c r="J16" s="1">
+        <v>0</v>
+      </c>
+      <c r="K16" s="1">
+        <v>0</v>
+      </c>
+      <c r="L16" s="1">
+        <v>1</v>
+      </c>
+      <c r="M16" s="1">
+        <v>0</v>
+      </c>
+      <c r="O16" s="1">
+        <f>A5</f>
+        <v>0</v>
+      </c>
+      <c r="P16" s="1">
+        <f>B5</f>
+        <v>1</v>
+      </c>
+      <c r="Q16" s="1">
+        <f>C5</f>
+        <v>0</v>
+      </c>
+      <c r="R16" s="1">
+        <f>D5</f>
+        <v>0</v>
+      </c>
+      <c r="S16" s="1">
+        <f>E5</f>
+        <v>1</v>
+      </c>
+      <c r="T16" s="1">
+        <f>F5</f>
+        <v>0</v>
+      </c>
+      <c r="V16" s="4">
         <v>1.907485954219941e-05</v>
       </c>
-      <c r="B16" s="4">
+      <c r="W16" s="4">
         <v>0.99999244565144241</v>
       </c>
-      <c r="C16" s="4">
+      <c r="X16" s="4">
         <v>0.00037878348203297511</v>
       </c>
-      <c r="D16" s="4">
+      <c r="Y16" s="4">
         <v>0.00013462097945892448</v>
       </c>
-      <c r="E16" s="4">
+      <c r="Z16" s="4">
         <v>0.99966391310430336</v>
       </c>
-      <c r="F16" s="4">
+      <c r="AA16" s="4">
         <v>2.1781724983351263e-05</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4">
+      <c r="A17" s="1">
+        <v>0</v>
+      </c>
+      <c r="B17" s="1">
+        <v>1</v>
+      </c>
+      <c r="C17" s="1">
+        <v>0</v>
+      </c>
+      <c r="D17" s="1">
+        <v>0</v>
+      </c>
+      <c r="E17" s="1">
+        <v>1</v>
+      </c>
+      <c r="F17" s="1">
+        <v>0</v>
+      </c>
+      <c r="H17" s="1">
+        <v>0</v>
+      </c>
+      <c r="I17" s="1">
+        <v>1</v>
+      </c>
+      <c r="J17" s="1">
+        <v>0</v>
+      </c>
+      <c r="K17" s="1">
+        <v>0</v>
+      </c>
+      <c r="L17" s="1">
+        <v>1</v>
+      </c>
+      <c r="M17" s="1">
+        <v>0</v>
+      </c>
+      <c r="O17" s="1">
+        <f>A6</f>
+        <v>0</v>
+      </c>
+      <c r="P17" s="1">
+        <f>B6</f>
+        <v>1</v>
+      </c>
+      <c r="Q17" s="1">
+        <f>C6</f>
+        <v>0</v>
+      </c>
+      <c r="R17" s="1">
+        <f>D6</f>
+        <v>0</v>
+      </c>
+      <c r="S17" s="1">
+        <f>E6</f>
+        <v>1</v>
+      </c>
+      <c r="T17" s="1">
+        <f>F6</f>
+        <v>0</v>
+      </c>
+      <c r="V17" s="4">
         <v>1.1467554001383744e-05</v>
       </c>
-      <c r="B17" s="4">
+      <c r="W17" s="4">
         <v>0.99995641206828578</v>
       </c>
-      <c r="C17" s="4">
+      <c r="X17" s="4">
         <v>2.0156208110510332e-05</v>
       </c>
-      <c r="D17" s="4">
+      <c r="Y17" s="4">
         <v>8.3438085639179678e-08</v>
       </c>
-      <c r="E17" s="4">
+      <c r="Z17" s="4">
         <v>0.99999963867424579</v>
       </c>
-      <c r="F17" s="4">
+      <c r="AA17" s="4">
         <v>2.7592302018243459e-05</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4">
+      <c r="A18" s="1">
+        <v>0</v>
+      </c>
+      <c r="B18" s="1">
+        <v>0</v>
+      </c>
+      <c r="C18" s="1">
+        <v>1</v>
+      </c>
+      <c r="D18" s="1">
+        <v>1</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0</v>
+      </c>
+      <c r="F18" s="1">
+        <v>0</v>
+      </c>
+      <c r="H18" s="1">
+        <v>0</v>
+      </c>
+      <c r="I18" s="1">
+        <v>0</v>
+      </c>
+      <c r="J18" s="1">
+        <v>1</v>
+      </c>
+      <c r="K18" s="1">
+        <v>1</v>
+      </c>
+      <c r="L18" s="1">
+        <v>0</v>
+      </c>
+      <c r="M18" s="1">
+        <v>0</v>
+      </c>
+      <c r="O18" s="1">
+        <f>A7</f>
+        <v>0</v>
+      </c>
+      <c r="P18" s="1">
+        <f>B7</f>
+        <v>0</v>
+      </c>
+      <c r="Q18" s="1">
+        <f>C7</f>
+        <v>1</v>
+      </c>
+      <c r="R18" s="1">
+        <f>D7</f>
+        <v>1</v>
+      </c>
+      <c r="S18" s="1">
+        <f>E7</f>
+        <v>0</v>
+      </c>
+      <c r="T18" s="1">
+        <f>F7</f>
+        <v>0</v>
+      </c>
+      <c r="V18" s="4">
         <v>1.5494613333452739e-05</v>
       </c>
-      <c r="B18" s="4">
+      <c r="W18" s="4">
         <v>9.4138124302250981e-08</v>
       </c>
-      <c r="C18" s="4">
+      <c r="X18" s="4">
         <v>0.99994553632589278</v>
       </c>
-      <c r="D18" s="4">
+      <c r="Y18" s="4">
         <v>0.99993969100460867</v>
       </c>
-      <c r="E18" s="4">
+      <c r="Z18" s="4">
         <v>4.3878870587798194e-06</v>
       </c>
-      <c r="F18" s="4">
+      <c r="AA18" s="4">
         <v>1.6807576768635771e-05</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4">
+      <c r="A19" s="1">
+        <v>0</v>
+      </c>
+      <c r="B19" s="1">
+        <v>0</v>
+      </c>
+      <c r="C19" s="1">
+        <v>0</v>
+      </c>
+      <c r="D19" s="1">
+        <v>0</v>
+      </c>
+      <c r="E19" s="1">
+        <v>0</v>
+      </c>
+      <c r="F19" s="1">
+        <v>0</v>
+      </c>
+      <c r="H19" s="1">
+        <v>0</v>
+      </c>
+      <c r="I19" s="1">
+        <v>0</v>
+      </c>
+      <c r="J19" s="1">
+        <v>0</v>
+      </c>
+      <c r="K19" s="1">
+        <v>0</v>
+      </c>
+      <c r="L19" s="1">
+        <v>0</v>
+      </c>
+      <c r="M19" s="1">
+        <v>0</v>
+      </c>
+      <c r="O19" s="1">
+        <f>A8</f>
+        <v>0</v>
+      </c>
+      <c r="P19" s="1">
+        <f>B8</f>
+        <v>0</v>
+      </c>
+      <c r="Q19" s="1">
+        <f>C8</f>
+        <v>0</v>
+      </c>
+      <c r="R19" s="1">
+        <f>D8</f>
+        <v>0</v>
+      </c>
+      <c r="S19" s="1">
+        <f>E8</f>
+        <v>0</v>
+      </c>
+      <c r="T19" s="1">
+        <f>F8</f>
+        <v>0</v>
+      </c>
+      <c r="V19" s="4">
         <v>1.9330154764318981e-05</v>
       </c>
-      <c r="B19" s="4">
+      <c r="W19" s="4">
         <v>2.3990782687724591e-05</v>
       </c>
-      <c r="C19" s="4">
+      <c r="X19" s="4">
         <v>3.4588674630739308e-05</v>
       </c>
-      <c r="D19" s="4">
+      <c r="Y19" s="4">
         <v>1.8716269144037574e-05</v>
       </c>
-      <c r="E19" s="4">
+      <c r="Z19" s="4">
         <v>2.7860037933183034e-05</v>
       </c>
-      <c r="F19" s="4">
+      <c r="AA19" s="4">
         <v>1.8721410404438209e-05</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:F8 H1:BC1">
+  <conditionalFormatting sqref="A1:F8 H1:BC1 A12:F19 H12:M19 O12:T19">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThanOrEqual">
       <formula>0.5</formula>
     </cfRule>
@@ -1298,7 +2288,7 @@
       <formula>0.5</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A12:F19">
+  <conditionalFormatting sqref="V12:AA19">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -1680,7 +2670,7 @@
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t>A12:F19: probabilidades antes do limiar, em escala de cores fixa de 0 a 1.</t>
+          <t>Linha 12, lado a lado: matrizes originais, resultado e probabilidades antes do limiar.</t>
         </is>
       </c>
     </row>
@@ -1717,174 +2707,669 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="0" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Original 0 (A)</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Original 8 (B)</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>Resultado</t>
+        </is>
+      </c>
+      <c r="V11" s="5" t="inlineStr">
         <is>
           <t>Probabilidades</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4">
+      <c r="A12" s="1">
+        <v>0</v>
+      </c>
+      <c r="B12" s="1">
+        <v>0</v>
+      </c>
+      <c r="C12" s="1">
+        <v>0</v>
+      </c>
+      <c r="D12" s="1">
+        <v>0</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0</v>
+      </c>
+      <c r="F12" s="1">
+        <v>0</v>
+      </c>
+      <c r="H12" s="1">
+        <v>0</v>
+      </c>
+      <c r="I12" s="1">
+        <v>0</v>
+      </c>
+      <c r="J12" s="1">
+        <v>0</v>
+      </c>
+      <c r="K12" s="1">
+        <v>0</v>
+      </c>
+      <c r="L12" s="1">
+        <v>0</v>
+      </c>
+      <c r="M12" s="1">
+        <v>0</v>
+      </c>
+      <c r="O12" s="1">
+        <f>A1</f>
+        <v>0</v>
+      </c>
+      <c r="P12" s="1">
+        <f>B1</f>
+        <v>0</v>
+      </c>
+      <c r="Q12" s="1">
+        <f>C1</f>
+        <v>0</v>
+      </c>
+      <c r="R12" s="1">
+        <f>D1</f>
+        <v>0</v>
+      </c>
+      <c r="S12" s="1">
+        <f>E1</f>
+        <v>0</v>
+      </c>
+      <c r="T12" s="1">
+        <f>F1</f>
+        <v>0</v>
+      </c>
+      <c r="V12" s="4">
         <v>3.3084461954320121e-06</v>
       </c>
-      <c r="B12" s="4">
+      <c r="W12" s="4">
         <v>2.5316372855678328e-06</v>
       </c>
-      <c r="C12" s="4">
+      <c r="X12" s="4">
         <v>3.1733619139645755e-06</v>
       </c>
-      <c r="D12" s="4">
+      <c r="Y12" s="4">
         <v>1.9318540615750416e-06</v>
       </c>
-      <c r="E12" s="4">
+      <c r="Z12" s="4">
         <v>3.8321772697448748e-06</v>
       </c>
-      <c r="F12" s="4">
+      <c r="AA12" s="4">
         <v>1.8881535784373963e-06</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4">
+      <c r="A13" s="1">
+        <v>0</v>
+      </c>
+      <c r="B13" s="1">
+        <v>0</v>
+      </c>
+      <c r="C13" s="1">
+        <v>1</v>
+      </c>
+      <c r="D13" s="1">
+        <v>1</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0</v>
+      </c>
+      <c r="H13" s="1">
+        <v>0</v>
+      </c>
+      <c r="I13" s="1">
+        <v>0</v>
+      </c>
+      <c r="J13" s="1">
+        <v>1</v>
+      </c>
+      <c r="K13" s="1">
+        <v>1</v>
+      </c>
+      <c r="L13" s="1">
+        <v>0</v>
+      </c>
+      <c r="M13" s="1">
+        <v>0</v>
+      </c>
+      <c r="O13" s="1">
+        <f>A2</f>
+        <v>0</v>
+      </c>
+      <c r="P13" s="1">
+        <f>B2</f>
+        <v>0</v>
+      </c>
+      <c r="Q13" s="1">
+        <f>C2</f>
+        <v>1</v>
+      </c>
+      <c r="R13" s="1">
+        <f>D2</f>
+        <v>1</v>
+      </c>
+      <c r="S13" s="1">
+        <f>E2</f>
+        <v>0</v>
+      </c>
+      <c r="T13" s="1">
+        <f>F2</f>
+        <v>0</v>
+      </c>
+      <c r="V13" s="4">
         <v>1.2090273716224556e-06</v>
       </c>
-      <c r="B13" s="4">
+      <c r="W13" s="4">
         <v>1.5981070248291073e-05</v>
       </c>
-      <c r="C13" s="4">
+      <c r="X13" s="4">
         <v>0.99999996073586406</v>
       </c>
-      <c r="D13" s="4">
+      <c r="Y13" s="4">
         <v>0.99999977350002545</v>
       </c>
-      <c r="E13" s="4">
+      <c r="Z13" s="4">
         <v>1.0820045458774223e-05</v>
       </c>
-      <c r="F13" s="4">
+      <c r="AA13" s="4">
         <v>2.8046201979260223e-06</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4">
+      <c r="A14" s="1">
+        <v>0</v>
+      </c>
+      <c r="B14" s="1">
+        <v>1</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1">
+        <v>1</v>
+      </c>
+      <c r="F14" s="1">
+        <v>0</v>
+      </c>
+      <c r="H14" s="1">
+        <v>0</v>
+      </c>
+      <c r="I14" s="1">
+        <v>1</v>
+      </c>
+      <c r="J14" s="1">
+        <v>0</v>
+      </c>
+      <c r="K14" s="1">
+        <v>0</v>
+      </c>
+      <c r="L14" s="1">
+        <v>1</v>
+      </c>
+      <c r="M14" s="1">
+        <v>0</v>
+      </c>
+      <c r="O14" s="1">
+        <f>A3</f>
+        <v>0</v>
+      </c>
+      <c r="P14" s="1">
+        <f>B3</f>
+        <v>1</v>
+      </c>
+      <c r="Q14" s="1">
+        <f>C3</f>
+        <v>0</v>
+      </c>
+      <c r="R14" s="1">
+        <f>D3</f>
+        <v>0</v>
+      </c>
+      <c r="S14" s="1">
+        <f>E3</f>
+        <v>1</v>
+      </c>
+      <c r="T14" s="1">
+        <f>F3</f>
+        <v>0</v>
+      </c>
+      <c r="V14" s="4">
         <v>2.1446737450186787e-06</v>
       </c>
-      <c r="B14" s="4">
+      <c r="W14" s="4">
         <v>0.99999965825783743</v>
       </c>
-      <c r="C14" s="4">
+      <c r="X14" s="4">
         <v>1.0031023918817212e-07</v>
       </c>
-      <c r="D14" s="4">
+      <c r="Y14" s="4">
         <v>2.2090954148541462e-08</v>
       </c>
-      <c r="E14" s="4">
+      <c r="Z14" s="4">
         <v>0.99999970926888693</v>
       </c>
-      <c r="F14" s="4">
+      <c r="AA14" s="4">
         <v>8.8940371974996588e-07</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4">
+      <c r="A15" s="1">
+        <v>0</v>
+      </c>
+      <c r="B15" s="1">
+        <v>1</v>
+      </c>
+      <c r="C15" s="1">
+        <v>0</v>
+      </c>
+      <c r="D15" s="1">
+        <v>0</v>
+      </c>
+      <c r="E15" s="1">
+        <v>1</v>
+      </c>
+      <c r="F15" s="1">
+        <v>0</v>
+      </c>
+      <c r="H15" s="1">
+        <v>0</v>
+      </c>
+      <c r="I15" s="1">
+        <v>0</v>
+      </c>
+      <c r="J15" s="1">
+        <v>1</v>
+      </c>
+      <c r="K15" s="1">
+        <v>1</v>
+      </c>
+      <c r="L15" s="1">
+        <v>0</v>
+      </c>
+      <c r="M15" s="1">
+        <v>0</v>
+      </c>
+      <c r="O15" s="1">
+        <f>A4</f>
+        <v>0</v>
+      </c>
+      <c r="P15" s="1">
+        <f>B4</f>
+        <v>0</v>
+      </c>
+      <c r="Q15" s="1">
+        <f>C4</f>
+        <v>1</v>
+      </c>
+      <c r="R15" s="1">
+        <f>D4</f>
+        <v>1</v>
+      </c>
+      <c r="S15" s="1">
+        <f>E4</f>
+        <v>0</v>
+      </c>
+      <c r="T15" s="1">
+        <f>F4</f>
+        <v>0</v>
+      </c>
+      <c r="V15" s="4">
         <v>8.4961098018982528e-07</v>
       </c>
-      <c r="B15" s="4">
+      <c r="W15" s="4">
         <v>0.14556628984343287</v>
       </c>
-      <c r="C15" s="4">
+      <c r="X15" s="4">
         <v>0.87290295383400174</v>
       </c>
-      <c r="D15" s="4">
+      <c r="Y15" s="4">
         <v>0.85188042176231593</v>
       </c>
-      <c r="E15" s="4">
+      <c r="Z15" s="4">
         <v>0.38771266109485208</v>
       </c>
-      <c r="F15" s="4">
+      <c r="AA15" s="4">
         <v>1.3310575989257066e-06</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4">
+      <c r="A16" s="1">
+        <v>0</v>
+      </c>
+      <c r="B16" s="1">
+        <v>1</v>
+      </c>
+      <c r="C16" s="1">
+        <v>0</v>
+      </c>
+      <c r="D16" s="1">
+        <v>0</v>
+      </c>
+      <c r="E16" s="1">
+        <v>1</v>
+      </c>
+      <c r="F16" s="1">
+        <v>0</v>
+      </c>
+      <c r="H16" s="1">
+        <v>0</v>
+      </c>
+      <c r="I16" s="1">
+        <v>1</v>
+      </c>
+      <c r="J16" s="1">
+        <v>0</v>
+      </c>
+      <c r="K16" s="1">
+        <v>0</v>
+      </c>
+      <c r="L16" s="1">
+        <v>1</v>
+      </c>
+      <c r="M16" s="1">
+        <v>0</v>
+      </c>
+      <c r="O16" s="1">
+        <f>A5</f>
+        <v>0</v>
+      </c>
+      <c r="P16" s="1">
+        <f>B5</f>
+        <v>1</v>
+      </c>
+      <c r="Q16" s="1">
+        <f>C5</f>
+        <v>0</v>
+      </c>
+      <c r="R16" s="1">
+        <f>D5</f>
+        <v>0</v>
+      </c>
+      <c r="S16" s="1">
+        <f>E5</f>
+        <v>1</v>
+      </c>
+      <c r="T16" s="1">
+        <f>F5</f>
+        <v>0</v>
+      </c>
+      <c r="V16" s="4">
         <v>1.4979055911488175e-06</v>
       </c>
-      <c r="B16" s="4">
+      <c r="W16" s="4">
         <v>0.99983483501861004</v>
       </c>
-      <c r="C16" s="4">
+      <c r="X16" s="4">
         <v>1.7770616964646277e-05</v>
       </c>
-      <c r="D16" s="4">
+      <c r="Y16" s="4">
         <v>2.0752013526479602e-06</v>
       </c>
-      <c r="E16" s="4">
+      <c r="Z16" s="4">
         <v>0.99957906092258386</v>
       </c>
-      <c r="F16" s="4">
+      <c r="AA16" s="4">
         <v>1.8602982164520343e-06</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4">
+      <c r="A17" s="1">
+        <v>0</v>
+      </c>
+      <c r="B17" s="1">
+        <v>1</v>
+      </c>
+      <c r="C17" s="1">
+        <v>0</v>
+      </c>
+      <c r="D17" s="1">
+        <v>0</v>
+      </c>
+      <c r="E17" s="1">
+        <v>1</v>
+      </c>
+      <c r="F17" s="1">
+        <v>0</v>
+      </c>
+      <c r="H17" s="1">
+        <v>0</v>
+      </c>
+      <c r="I17" s="1">
+        <v>1</v>
+      </c>
+      <c r="J17" s="1">
+        <v>0</v>
+      </c>
+      <c r="K17" s="1">
+        <v>0</v>
+      </c>
+      <c r="L17" s="1">
+        <v>1</v>
+      </c>
+      <c r="M17" s="1">
+        <v>0</v>
+      </c>
+      <c r="O17" s="1">
+        <f>A6</f>
+        <v>0</v>
+      </c>
+      <c r="P17" s="1">
+        <f>B6</f>
+        <v>1</v>
+      </c>
+      <c r="Q17" s="1">
+        <f>C6</f>
+        <v>0</v>
+      </c>
+      <c r="R17" s="1">
+        <f>D6</f>
+        <v>0</v>
+      </c>
+      <c r="S17" s="1">
+        <f>E6</f>
+        <v>1</v>
+      </c>
+      <c r="T17" s="1">
+        <f>F6</f>
+        <v>0</v>
+      </c>
+      <c r="V17" s="4">
         <v>9.4259904315785698e-07</v>
       </c>
-      <c r="B17" s="4">
+      <c r="W17" s="4">
         <v>0.99986678511356963</v>
       </c>
-      <c r="C17" s="4">
+      <c r="X17" s="4">
         <v>1.6977120702804035e-06</v>
       </c>
-      <c r="D17" s="4">
+      <c r="Y17" s="4">
         <v>6.0598715444115531e-08</v>
       </c>
-      <c r="E17" s="4">
+      <c r="Z17" s="4">
         <v>0.99998758839904933</v>
       </c>
-      <c r="F17" s="4">
+      <c r="AA17" s="4">
         <v>3.5471103168817635e-06</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4">
+      <c r="A18" s="1">
+        <v>0</v>
+      </c>
+      <c r="B18" s="1">
+        <v>0</v>
+      </c>
+      <c r="C18" s="1">
+        <v>1</v>
+      </c>
+      <c r="D18" s="1">
+        <v>1</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0</v>
+      </c>
+      <c r="F18" s="1">
+        <v>0</v>
+      </c>
+      <c r="H18" s="1">
+        <v>0</v>
+      </c>
+      <c r="I18" s="1">
+        <v>0</v>
+      </c>
+      <c r="J18" s="1">
+        <v>1</v>
+      </c>
+      <c r="K18" s="1">
+        <v>1</v>
+      </c>
+      <c r="L18" s="1">
+        <v>0</v>
+      </c>
+      <c r="M18" s="1">
+        <v>0</v>
+      </c>
+      <c r="O18" s="1">
+        <f>A7</f>
+        <v>0</v>
+      </c>
+      <c r="P18" s="1">
+        <f>B7</f>
+        <v>0</v>
+      </c>
+      <c r="Q18" s="1">
+        <f>C7</f>
+        <v>1</v>
+      </c>
+      <c r="R18" s="1">
+        <f>D7</f>
+        <v>1</v>
+      </c>
+      <c r="S18" s="1">
+        <f>E7</f>
+        <v>0</v>
+      </c>
+      <c r="T18" s="1">
+        <f>F7</f>
+        <v>0</v>
+      </c>
+      <c r="V18" s="4">
         <v>1.1694882505078095e-06</v>
       </c>
-      <c r="B18" s="4">
+      <c r="W18" s="4">
         <v>8.9431108406162608e-06</v>
       </c>
-      <c r="C18" s="4">
+      <c r="X18" s="4">
         <v>0.99999848796437296</v>
       </c>
-      <c r="D18" s="4">
+      <c r="Y18" s="4">
         <v>0.99999848618549214</v>
       </c>
-      <c r="E18" s="4">
+      <c r="Z18" s="4">
         <v>1.9645841899796831e-05</v>
       </c>
-      <c r="F18" s="4">
+      <c r="AA18" s="4">
         <v>1.6776337793871725e-06</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4">
+      <c r="A19" s="1">
+        <v>0</v>
+      </c>
+      <c r="B19" s="1">
+        <v>0</v>
+      </c>
+      <c r="C19" s="1">
+        <v>0</v>
+      </c>
+      <c r="D19" s="1">
+        <v>0</v>
+      </c>
+      <c r="E19" s="1">
+        <v>0</v>
+      </c>
+      <c r="F19" s="1">
+        <v>0</v>
+      </c>
+      <c r="H19" s="1">
+        <v>0</v>
+      </c>
+      <c r="I19" s="1">
+        <v>0</v>
+      </c>
+      <c r="J19" s="1">
+        <v>0</v>
+      </c>
+      <c r="K19" s="1">
+        <v>0</v>
+      </c>
+      <c r="L19" s="1">
+        <v>0</v>
+      </c>
+      <c r="M19" s="1">
+        <v>0</v>
+      </c>
+      <c r="O19" s="1">
+        <f>A8</f>
+        <v>0</v>
+      </c>
+      <c r="P19" s="1">
+        <f>B8</f>
+        <v>0</v>
+      </c>
+      <c r="Q19" s="1">
+        <f>C8</f>
+        <v>0</v>
+      </c>
+      <c r="R19" s="1">
+        <f>D8</f>
+        <v>0</v>
+      </c>
+      <c r="S19" s="1">
+        <f>E8</f>
+        <v>0</v>
+      </c>
+      <c r="T19" s="1">
+        <f>F8</f>
+        <v>0</v>
+      </c>
+      <c r="V19" s="4">
         <v>1.5156225347315332e-06</v>
       </c>
-      <c r="B19" s="4">
+      <c r="W19" s="4">
         <v>2.2770785463418935e-06</v>
       </c>
-      <c r="C19" s="4">
+      <c r="X19" s="4">
         <v>2.9881563124482498e-06</v>
       </c>
-      <c r="D19" s="4">
+      <c r="Y19" s="4">
         <v>1.6545038777405503e-06</v>
       </c>
-      <c r="E19" s="4">
+      <c r="Z19" s="4">
         <v>2.5476037480352035e-06</v>
       </c>
-      <c r="F19" s="4">
+      <c r="AA19" s="4">
         <v>1.5453612690510687e-06</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:F8 H1:BC1">
+  <conditionalFormatting sqref="A1:F8 H1:BC1 A12:F19 H12:M19 O12:T19">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThanOrEqual">
       <formula>0.5</formula>
     </cfRule>
@@ -1892,7 +3377,7 @@
       <formula>0.5</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A12:F19">
+  <conditionalFormatting sqref="V12:AA19">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -2274,7 +3759,7 @@
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t>A12:F19: probabilidades antes do limiar, em escala de cores fixa de 0 a 1.</t>
+          <t>Linha 12, lado a lado: matrizes originais, resultado e probabilidades antes do limiar.</t>
         </is>
       </c>
     </row>
@@ -2311,174 +3796,669 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="0" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Original 0 (A)</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Original 8 (B)</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>Resultado</t>
+        </is>
+      </c>
+      <c r="V11" s="5" t="inlineStr">
         <is>
           <t>Probabilidades</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4">
+      <c r="A12" s="1">
+        <v>0</v>
+      </c>
+      <c r="B12" s="1">
+        <v>0</v>
+      </c>
+      <c r="C12" s="1">
+        <v>0</v>
+      </c>
+      <c r="D12" s="1">
+        <v>0</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0</v>
+      </c>
+      <c r="F12" s="1">
+        <v>0</v>
+      </c>
+      <c r="H12" s="1">
+        <v>0</v>
+      </c>
+      <c r="I12" s="1">
+        <v>0</v>
+      </c>
+      <c r="J12" s="1">
+        <v>0</v>
+      </c>
+      <c r="K12" s="1">
+        <v>0</v>
+      </c>
+      <c r="L12" s="1">
+        <v>0</v>
+      </c>
+      <c r="M12" s="1">
+        <v>0</v>
+      </c>
+      <c r="O12" s="1">
+        <f>A1</f>
+        <v>0</v>
+      </c>
+      <c r="P12" s="1">
+        <f>B1</f>
+        <v>0</v>
+      </c>
+      <c r="Q12" s="1">
+        <f>C1</f>
+        <v>0</v>
+      </c>
+      <c r="R12" s="1">
+        <f>D1</f>
+        <v>0</v>
+      </c>
+      <c r="S12" s="1">
+        <f>E1</f>
+        <v>0</v>
+      </c>
+      <c r="T12" s="1">
+        <f>F1</f>
+        <v>0</v>
+      </c>
+      <c r="V12" s="4">
         <v>1.9235478136818721e-06</v>
       </c>
-      <c r="B12" s="4">
+      <c r="W12" s="4">
         <v>9.6457447236685482e-07</v>
       </c>
-      <c r="C12" s="4">
+      <c r="X12" s="4">
         <v>1.8644160628046895e-06</v>
       </c>
-      <c r="D12" s="4">
+      <c r="Y12" s="4">
         <v>8.638508650249599e-07</v>
       </c>
-      <c r="E12" s="4">
+      <c r="Z12" s="4">
         <v>1.7700972579263787e-06</v>
       </c>
-      <c r="F12" s="4">
+      <c r="AA12" s="4">
         <v>7.5654668385996578e-07</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4">
+      <c r="A13" s="1">
+        <v>0</v>
+      </c>
+      <c r="B13" s="1">
+        <v>0</v>
+      </c>
+      <c r="C13" s="1">
+        <v>1</v>
+      </c>
+      <c r="D13" s="1">
+        <v>1</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0</v>
+      </c>
+      <c r="H13" s="1">
+        <v>0</v>
+      </c>
+      <c r="I13" s="1">
+        <v>0</v>
+      </c>
+      <c r="J13" s="1">
+        <v>1</v>
+      </c>
+      <c r="K13" s="1">
+        <v>1</v>
+      </c>
+      <c r="L13" s="1">
+        <v>0</v>
+      </c>
+      <c r="M13" s="1">
+        <v>0</v>
+      </c>
+      <c r="O13" s="1">
+        <f>A2</f>
+        <v>0</v>
+      </c>
+      <c r="P13" s="1">
+        <f>B2</f>
+        <v>0</v>
+      </c>
+      <c r="Q13" s="1">
+        <f>C2</f>
+        <v>1</v>
+      </c>
+      <c r="R13" s="1">
+        <f>D2</f>
+        <v>1</v>
+      </c>
+      <c r="S13" s="1">
+        <f>E2</f>
+        <v>0</v>
+      </c>
+      <c r="T13" s="1">
+        <f>F2</f>
+        <v>0</v>
+      </c>
+      <c r="V13" s="4">
         <v>4.1766085175550729e-07</v>
       </c>
-      <c r="B13" s="4">
+      <c r="W13" s="4">
         <v>4.6412353219689089e-05</v>
       </c>
-      <c r="C13" s="4">
+      <c r="X13" s="4">
         <v>0.99999999210920743</v>
       </c>
-      <c r="D13" s="4">
+      <c r="Y13" s="4">
         <v>0.9999999896956534</v>
       </c>
-      <c r="E13" s="4">
+      <c r="Z13" s="4">
         <v>4.2160039854155921e-05</v>
       </c>
-      <c r="F13" s="4">
+      <c r="AA13" s="4">
         <v>1.0689513376782598e-06</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4">
+      <c r="A14" s="1">
+        <v>0</v>
+      </c>
+      <c r="B14" s="1">
+        <v>1</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1">
+        <v>1</v>
+      </c>
+      <c r="F14" s="1">
+        <v>0</v>
+      </c>
+      <c r="H14" s="1">
+        <v>0</v>
+      </c>
+      <c r="I14" s="1">
+        <v>1</v>
+      </c>
+      <c r="J14" s="1">
+        <v>0</v>
+      </c>
+      <c r="K14" s="1">
+        <v>0</v>
+      </c>
+      <c r="L14" s="1">
+        <v>1</v>
+      </c>
+      <c r="M14" s="1">
+        <v>0</v>
+      </c>
+      <c r="O14" s="1">
+        <f>A3</f>
+        <v>0</v>
+      </c>
+      <c r="P14" s="1">
+        <f>B3</f>
+        <v>1</v>
+      </c>
+      <c r="Q14" s="1">
+        <f>C3</f>
+        <v>0</v>
+      </c>
+      <c r="R14" s="1">
+        <f>D3</f>
+        <v>0</v>
+      </c>
+      <c r="S14" s="1">
+        <f>E3</f>
+        <v>1</v>
+      </c>
+      <c r="T14" s="1">
+        <f>F3</f>
+        <v>0</v>
+      </c>
+      <c r="V14" s="4">
         <v>9.8935491577264783e-07</v>
       </c>
-      <c r="B14" s="4">
+      <c r="W14" s="4">
         <v>0.99999730482113103</v>
       </c>
-      <c r="C14" s="4">
+      <c r="X14" s="4">
         <v>1.2467708436142754e-07</v>
       </c>
-      <c r="D14" s="4">
+      <c r="Y14" s="4">
         <v>1.9944127678530483e-07</v>
       </c>
-      <c r="E14" s="4">
+      <c r="Z14" s="4">
         <v>0.99998992933314468</v>
       </c>
-      <c r="F14" s="4">
+      <c r="AA14" s="4">
         <v>3.0112064521816815e-07</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4">
+      <c r="A15" s="1">
+        <v>0</v>
+      </c>
+      <c r="B15" s="1">
+        <v>1</v>
+      </c>
+      <c r="C15" s="1">
+        <v>0</v>
+      </c>
+      <c r="D15" s="1">
+        <v>0</v>
+      </c>
+      <c r="E15" s="1">
+        <v>1</v>
+      </c>
+      <c r="F15" s="1">
+        <v>0</v>
+      </c>
+      <c r="H15" s="1">
+        <v>0</v>
+      </c>
+      <c r="I15" s="1">
+        <v>0</v>
+      </c>
+      <c r="J15" s="1">
+        <v>1</v>
+      </c>
+      <c r="K15" s="1">
+        <v>1</v>
+      </c>
+      <c r="L15" s="1">
+        <v>0</v>
+      </c>
+      <c r="M15" s="1">
+        <v>0</v>
+      </c>
+      <c r="O15" s="1">
+        <f>A4</f>
+        <v>0</v>
+      </c>
+      <c r="P15" s="1">
+        <f>B4</f>
+        <v>0</v>
+      </c>
+      <c r="Q15" s="1">
+        <f>C4</f>
+        <v>1</v>
+      </c>
+      <c r="R15" s="1">
+        <f>D4</f>
+        <v>1</v>
+      </c>
+      <c r="S15" s="1">
+        <f>E4</f>
+        <v>0</v>
+      </c>
+      <c r="T15" s="1">
+        <f>F4</f>
+        <v>0</v>
+      </c>
+      <c r="V15" s="4">
         <v>2.6441611985357139e-07</v>
       </c>
-      <c r="B15" s="4">
+      <c r="W15" s="4">
         <v>0.0010589407022586624</v>
       </c>
-      <c r="C15" s="4">
+      <c r="X15" s="4">
         <v>0.99952104476889292</v>
       </c>
-      <c r="D15" s="4">
+      <c r="Y15" s="4">
         <v>0.9991180389161417</v>
       </c>
-      <c r="E15" s="4">
+      <c r="Z15" s="4">
         <v>0.0044216832284960789</v>
       </c>
-      <c r="F15" s="4">
+      <c r="AA15" s="4">
         <v>4.850646546692811e-07</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4">
+      <c r="A16" s="1">
+        <v>0</v>
+      </c>
+      <c r="B16" s="1">
+        <v>1</v>
+      </c>
+      <c r="C16" s="1">
+        <v>0</v>
+      </c>
+      <c r="D16" s="1">
+        <v>0</v>
+      </c>
+      <c r="E16" s="1">
+        <v>1</v>
+      </c>
+      <c r="F16" s="1">
+        <v>0</v>
+      </c>
+      <c r="H16" s="1">
+        <v>0</v>
+      </c>
+      <c r="I16" s="1">
+        <v>1</v>
+      </c>
+      <c r="J16" s="1">
+        <v>0</v>
+      </c>
+      <c r="K16" s="1">
+        <v>0</v>
+      </c>
+      <c r="L16" s="1">
+        <v>1</v>
+      </c>
+      <c r="M16" s="1">
+        <v>0</v>
+      </c>
+      <c r="O16" s="1">
+        <f>A5</f>
+        <v>0</v>
+      </c>
+      <c r="P16" s="1">
+        <f>B5</f>
+        <v>1</v>
+      </c>
+      <c r="Q16" s="1">
+        <f>C5</f>
+        <v>0</v>
+      </c>
+      <c r="R16" s="1">
+        <f>D5</f>
+        <v>0</v>
+      </c>
+      <c r="S16" s="1">
+        <f>E5</f>
+        <v>1</v>
+      </c>
+      <c r="T16" s="1">
+        <f>F5</f>
+        <v>0</v>
+      </c>
+      <c r="V16" s="4">
         <v>4.6750402798196055e-07</v>
       </c>
-      <c r="B16" s="4">
+      <c r="W16" s="4">
         <v>0.99921040440031361</v>
       </c>
-      <c r="C16" s="4">
+      <c r="X16" s="4">
         <v>1.6312095936876687e-06</v>
       </c>
-      <c r="D16" s="4">
+      <c r="Y16" s="4">
         <v>2.1791740771800402e-07</v>
       </c>
-      <c r="E16" s="4">
+      <c r="Z16" s="4">
         <v>0.99984818716140689</v>
       </c>
-      <c r="F16" s="4">
+      <c r="AA16" s="4">
         <v>6.6426304595585702e-07</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4">
+      <c r="A17" s="1">
+        <v>0</v>
+      </c>
+      <c r="B17" s="1">
+        <v>1</v>
+      </c>
+      <c r="C17" s="1">
+        <v>0</v>
+      </c>
+      <c r="D17" s="1">
+        <v>0</v>
+      </c>
+      <c r="E17" s="1">
+        <v>1</v>
+      </c>
+      <c r="F17" s="1">
+        <v>0</v>
+      </c>
+      <c r="H17" s="1">
+        <v>0</v>
+      </c>
+      <c r="I17" s="1">
+        <v>1</v>
+      </c>
+      <c r="J17" s="1">
+        <v>0</v>
+      </c>
+      <c r="K17" s="1">
+        <v>0</v>
+      </c>
+      <c r="L17" s="1">
+        <v>1</v>
+      </c>
+      <c r="M17" s="1">
+        <v>0</v>
+      </c>
+      <c r="O17" s="1">
+        <f>A6</f>
+        <v>0</v>
+      </c>
+      <c r="P17" s="1">
+        <f>B6</f>
+        <v>1</v>
+      </c>
+      <c r="Q17" s="1">
+        <f>C6</f>
+        <v>0</v>
+      </c>
+      <c r="R17" s="1">
+        <f>D6</f>
+        <v>0</v>
+      </c>
+      <c r="S17" s="1">
+        <f>E6</f>
+        <v>1</v>
+      </c>
+      <c r="T17" s="1">
+        <f>F6</f>
+        <v>0</v>
+      </c>
+      <c r="V17" s="4">
         <v>2.6917203065790582e-07</v>
       </c>
-      <c r="B17" s="4">
+      <c r="W17" s="4">
         <v>0.99908525315118601</v>
       </c>
-      <c r="C17" s="4">
+      <c r="X17" s="4">
         <v>6.5081329901684637e-07</v>
       </c>
-      <c r="D17" s="4">
+      <c r="Y17" s="4">
         <v>9.0775544840454656e-08</v>
       </c>
-      <c r="E17" s="4">
+      <c r="Z17" s="4">
         <v>0.99997209315774171</v>
       </c>
-      <c r="F17" s="4">
+      <c r="AA17" s="4">
         <v>1.3851649952373099e-06</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4">
+      <c r="A18" s="1">
+        <v>0</v>
+      </c>
+      <c r="B18" s="1">
+        <v>0</v>
+      </c>
+      <c r="C18" s="1">
+        <v>1</v>
+      </c>
+      <c r="D18" s="1">
+        <v>1</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0</v>
+      </c>
+      <c r="F18" s="1">
+        <v>0</v>
+      </c>
+      <c r="H18" s="1">
+        <v>0</v>
+      </c>
+      <c r="I18" s="1">
+        <v>0</v>
+      </c>
+      <c r="J18" s="1">
+        <v>1</v>
+      </c>
+      <c r="K18" s="1">
+        <v>1</v>
+      </c>
+      <c r="L18" s="1">
+        <v>0</v>
+      </c>
+      <c r="M18" s="1">
+        <v>0</v>
+      </c>
+      <c r="O18" s="1">
+        <f>A7</f>
+        <v>0</v>
+      </c>
+      <c r="P18" s="1">
+        <f>B7</f>
+        <v>0</v>
+      </c>
+      <c r="Q18" s="1">
+        <f>C7</f>
+        <v>1</v>
+      </c>
+      <c r="R18" s="1">
+        <f>D7</f>
+        <v>1</v>
+      </c>
+      <c r="S18" s="1">
+        <f>E7</f>
+        <v>0</v>
+      </c>
+      <c r="T18" s="1">
+        <f>F7</f>
+        <v>0</v>
+      </c>
+      <c r="V18" s="4">
         <v>4.060579667300621e-07</v>
       </c>
-      <c r="B18" s="4">
+      <c r="W18" s="4">
         <v>0.00010225375921406123</v>
       </c>
-      <c r="C18" s="4">
+      <c r="X18" s="4">
         <v>0.9999999132584485</v>
       </c>
-      <c r="D18" s="4">
+      <c r="Y18" s="4">
         <v>0.99999993318142644</v>
       </c>
-      <c r="E18" s="4">
+      <c r="Z18" s="4">
         <v>4.4524942788306052e-05</v>
       </c>
-      <c r="F18" s="4">
+      <c r="AA18" s="4">
         <v>6.8169754603389462e-07</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4">
+      <c r="A19" s="1">
+        <v>0</v>
+      </c>
+      <c r="B19" s="1">
+        <v>0</v>
+      </c>
+      <c r="C19" s="1">
+        <v>0</v>
+      </c>
+      <c r="D19" s="1">
+        <v>0</v>
+      </c>
+      <c r="E19" s="1">
+        <v>0</v>
+      </c>
+      <c r="F19" s="1">
+        <v>0</v>
+      </c>
+      <c r="H19" s="1">
+        <v>0</v>
+      </c>
+      <c r="I19" s="1">
+        <v>0</v>
+      </c>
+      <c r="J19" s="1">
+        <v>0</v>
+      </c>
+      <c r="K19" s="1">
+        <v>0</v>
+      </c>
+      <c r="L19" s="1">
+        <v>0</v>
+      </c>
+      <c r="M19" s="1">
+        <v>0</v>
+      </c>
+      <c r="O19" s="1">
+        <f>A8</f>
+        <v>0</v>
+      </c>
+      <c r="P19" s="1">
+        <f>B8</f>
+        <v>0</v>
+      </c>
+      <c r="Q19" s="1">
+        <f>C8</f>
+        <v>0</v>
+      </c>
+      <c r="R19" s="1">
+        <f>D8</f>
+        <v>0</v>
+      </c>
+      <c r="S19" s="1">
+        <f>E8</f>
+        <v>0</v>
+      </c>
+      <c r="T19" s="1">
+        <f>F8</f>
+        <v>0</v>
+      </c>
+      <c r="V19" s="4">
         <v>4.8670594432443066e-07</v>
       </c>
-      <c r="B19" s="4">
+      <c r="W19" s="4">
         <v>1.0494079531038043e-06</v>
       </c>
-      <c r="C19" s="4">
+      <c r="X19" s="4">
         <v>1.5032012536297669e-06</v>
       </c>
-      <c r="D19" s="4">
+      <c r="Y19" s="4">
         <v>6.2958137333882838e-07</v>
       </c>
-      <c r="E19" s="4">
+      <c r="Z19" s="4">
         <v>1.0194299848247141e-06</v>
       </c>
-      <c r="F19" s="4">
+      <c r="AA19" s="4">
         <v>5.8334202423811151e-07</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:F8 H1:BC1">
+  <conditionalFormatting sqref="A1:F8 H1:BC1 A12:F19 H12:M19 O12:T19">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThanOrEqual">
       <formula>0.5</formula>
     </cfRule>
@@ -2486,7 +4466,7 @@
       <formula>0.5</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A12:F19">
+  <conditionalFormatting sqref="V12:AA19">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -2868,7 +4848,7 @@
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t>A12:F19: probabilidades antes do limiar, em escala de cores fixa de 0 a 1.</t>
+          <t>Linha 12, lado a lado: matrizes originais, resultado e probabilidades antes do limiar.</t>
         </is>
       </c>
     </row>
@@ -2905,174 +4885,669 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="0" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Original 0 (A)</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Original 8 (B)</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>Resultado</t>
+        </is>
+      </c>
+      <c r="V11" s="5" t="inlineStr">
         <is>
           <t>Probabilidades</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4">
+      <c r="A12" s="1">
+        <v>0</v>
+      </c>
+      <c r="B12" s="1">
+        <v>0</v>
+      </c>
+      <c r="C12" s="1">
+        <v>0</v>
+      </c>
+      <c r="D12" s="1">
+        <v>0</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0</v>
+      </c>
+      <c r="F12" s="1">
+        <v>0</v>
+      </c>
+      <c r="H12" s="1">
+        <v>0</v>
+      </c>
+      <c r="I12" s="1">
+        <v>0</v>
+      </c>
+      <c r="J12" s="1">
+        <v>0</v>
+      </c>
+      <c r="K12" s="1">
+        <v>0</v>
+      </c>
+      <c r="L12" s="1">
+        <v>0</v>
+      </c>
+      <c r="M12" s="1">
+        <v>0</v>
+      </c>
+      <c r="O12" s="1">
+        <f>A1</f>
+        <v>0</v>
+      </c>
+      <c r="P12" s="1">
+        <f>B1</f>
+        <v>0</v>
+      </c>
+      <c r="Q12" s="1">
+        <f>C1</f>
+        <v>0</v>
+      </c>
+      <c r="R12" s="1">
+        <f>D1</f>
+        <v>0</v>
+      </c>
+      <c r="S12" s="1">
+        <f>E1</f>
+        <v>0</v>
+      </c>
+      <c r="T12" s="1">
+        <f>F1</f>
+        <v>0</v>
+      </c>
+      <c r="V12" s="4">
         <v>2.2991182264318483e-06</v>
       </c>
-      <c r="B12" s="4">
+      <c r="W12" s="4">
         <v>9.4908360076833444e-07</v>
       </c>
-      <c r="C12" s="4">
+      <c r="X12" s="4">
         <v>2.2546816569592904e-06</v>
       </c>
-      <c r="D12" s="4">
+      <c r="Y12" s="4">
         <v>9.4041539955851699e-07</v>
       </c>
-      <c r="E12" s="4">
+      <c r="Z12" s="4">
         <v>2.0243422949103569e-06</v>
       </c>
-      <c r="F12" s="4">
+      <c r="AA12" s="4">
         <v>8.3926878282541052e-07</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4">
+      <c r="A13" s="1">
+        <v>0</v>
+      </c>
+      <c r="B13" s="1">
+        <v>0</v>
+      </c>
+      <c r="C13" s="1">
+        <v>1</v>
+      </c>
+      <c r="D13" s="1">
+        <v>1</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0</v>
+      </c>
+      <c r="H13" s="1">
+        <v>0</v>
+      </c>
+      <c r="I13" s="1">
+        <v>0</v>
+      </c>
+      <c r="J13" s="1">
+        <v>1</v>
+      </c>
+      <c r="K13" s="1">
+        <v>1</v>
+      </c>
+      <c r="L13" s="1">
+        <v>0</v>
+      </c>
+      <c r="M13" s="1">
+        <v>0</v>
+      </c>
+      <c r="O13" s="1">
+        <f>A2</f>
+        <v>0</v>
+      </c>
+      <c r="P13" s="1">
+        <f>B2</f>
+        <v>0</v>
+      </c>
+      <c r="Q13" s="1">
+        <f>C2</f>
+        <v>1</v>
+      </c>
+      <c r="R13" s="1">
+        <f>D2</f>
+        <v>1</v>
+      </c>
+      <c r="S13" s="1">
+        <f>E2</f>
+        <v>0</v>
+      </c>
+      <c r="T13" s="1">
+        <f>F2</f>
+        <v>0</v>
+      </c>
+      <c r="V13" s="4">
         <v>4.0740976404820751e-07</v>
       </c>
-      <c r="B13" s="4">
+      <c r="W13" s="4">
         <v>6.9722734768411866e-05</v>
       </c>
-      <c r="C13" s="4">
+      <c r="X13" s="4">
         <v>0.999999992653132</v>
       </c>
-      <c r="D13" s="4">
+      <c r="Y13" s="4">
         <v>0.99999999253183247</v>
       </c>
-      <c r="E13" s="4">
+      <c r="Z13" s="4">
         <v>6.871379441466814e-05</v>
       </c>
-      <c r="F13" s="4">
+      <c r="AA13" s="4">
         <v>1.0439141885025886e-06</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4">
+      <c r="A14" s="1">
+        <v>0</v>
+      </c>
+      <c r="B14" s="1">
+        <v>1</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1">
+        <v>1</v>
+      </c>
+      <c r="F14" s="1">
+        <v>0</v>
+      </c>
+      <c r="H14" s="1">
+        <v>0</v>
+      </c>
+      <c r="I14" s="1">
+        <v>1</v>
+      </c>
+      <c r="J14" s="1">
+        <v>0</v>
+      </c>
+      <c r="K14" s="1">
+        <v>0</v>
+      </c>
+      <c r="L14" s="1">
+        <v>1</v>
+      </c>
+      <c r="M14" s="1">
+        <v>0</v>
+      </c>
+      <c r="O14" s="1">
+        <f>A3</f>
+        <v>0</v>
+      </c>
+      <c r="P14" s="1">
+        <f>B3</f>
+        <v>1</v>
+      </c>
+      <c r="Q14" s="1">
+        <f>C3</f>
+        <v>0</v>
+      </c>
+      <c r="R14" s="1">
+        <f>D3</f>
+        <v>0</v>
+      </c>
+      <c r="S14" s="1">
+        <f>E3</f>
+        <v>1</v>
+      </c>
+      <c r="T14" s="1">
+        <f>F3</f>
+        <v>0</v>
+      </c>
+      <c r="V14" s="4">
         <v>1.0612373412305877e-06</v>
       </c>
-      <c r="B14" s="4">
+      <c r="W14" s="4">
         <v>0.99999662152596958</v>
       </c>
-      <c r="C14" s="4">
+      <c r="X14" s="4">
         <v>1.3964046958760738e-07</v>
       </c>
-      <c r="D14" s="4">
+      <c r="Y14" s="4">
         <v>3.3772149391277048e-07</v>
       </c>
-      <c r="E14" s="4">
+      <c r="Z14" s="4">
         <v>0.9999758655458707</v>
       </c>
-      <c r="F14" s="4">
+      <c r="AA14" s="4">
         <v>3.0111043312990299e-07</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4">
+      <c r="A15" s="1">
+        <v>0</v>
+      </c>
+      <c r="B15" s="1">
+        <v>1</v>
+      </c>
+      <c r="C15" s="1">
+        <v>0</v>
+      </c>
+      <c r="D15" s="1">
+        <v>0</v>
+      </c>
+      <c r="E15" s="1">
+        <v>1</v>
+      </c>
+      <c r="F15" s="1">
+        <v>0</v>
+      </c>
+      <c r="H15" s="1">
+        <v>0</v>
+      </c>
+      <c r="I15" s="1">
+        <v>0</v>
+      </c>
+      <c r="J15" s="1">
+        <v>1</v>
+      </c>
+      <c r="K15" s="1">
+        <v>1</v>
+      </c>
+      <c r="L15" s="1">
+        <v>0</v>
+      </c>
+      <c r="M15" s="1">
+        <v>0</v>
+      </c>
+      <c r="O15" s="1">
+        <f>A4</f>
+        <v>0</v>
+      </c>
+      <c r="P15" s="1">
+        <f>B4</f>
+        <v>0</v>
+      </c>
+      <c r="Q15" s="1">
+        <f>C4</f>
+        <v>1</v>
+      </c>
+      <c r="R15" s="1">
+        <f>D4</f>
+        <v>1</v>
+      </c>
+      <c r="S15" s="1">
+        <f>E4</f>
+        <v>0</v>
+      </c>
+      <c r="T15" s="1">
+        <f>F4</f>
+        <v>0</v>
+      </c>
+      <c r="V15" s="4">
         <v>2.529346072626392e-07</v>
       </c>
-      <c r="B15" s="4">
+      <c r="W15" s="4">
         <v>0.00050441365389580935</v>
       </c>
-      <c r="C15" s="4">
+      <c r="X15" s="4">
         <v>0.99985104061702013</v>
       </c>
-      <c r="D15" s="4">
+      <c r="Y15" s="4">
         <v>0.99963767148537708</v>
       </c>
-      <c r="E15" s="4">
+      <c r="Z15" s="4">
         <v>0.0015071734592987515</v>
       </c>
-      <c r="F15" s="4">
+      <c r="AA15" s="4">
         <v>4.8481113278212083e-07</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4">
+      <c r="A16" s="1">
+        <v>0</v>
+      </c>
+      <c r="B16" s="1">
+        <v>1</v>
+      </c>
+      <c r="C16" s="1">
+        <v>0</v>
+      </c>
+      <c r="D16" s="1">
+        <v>0</v>
+      </c>
+      <c r="E16" s="1">
+        <v>1</v>
+      </c>
+      <c r="F16" s="1">
+        <v>0</v>
+      </c>
+      <c r="H16" s="1">
+        <v>0</v>
+      </c>
+      <c r="I16" s="1">
+        <v>1</v>
+      </c>
+      <c r="J16" s="1">
+        <v>0</v>
+      </c>
+      <c r="K16" s="1">
+        <v>0</v>
+      </c>
+      <c r="L16" s="1">
+        <v>1</v>
+      </c>
+      <c r="M16" s="1">
+        <v>0</v>
+      </c>
+      <c r="O16" s="1">
+        <f>A5</f>
+        <v>0</v>
+      </c>
+      <c r="P16" s="1">
+        <f>B5</f>
+        <v>1</v>
+      </c>
+      <c r="Q16" s="1">
+        <f>C5</f>
+        <v>0</v>
+      </c>
+      <c r="R16" s="1">
+        <f>D5</f>
+        <v>0</v>
+      </c>
+      <c r="S16" s="1">
+        <f>E5</f>
+        <v>1</v>
+      </c>
+      <c r="T16" s="1">
+        <f>F5</f>
+        <v>0</v>
+      </c>
+      <c r="V16" s="4">
         <v>4.6360137875823173e-07</v>
       </c>
-      <c r="B16" s="4">
+      <c r="W16" s="4">
         <v>0.99931635943740316</v>
       </c>
-      <c r="C16" s="4">
+      <c r="X16" s="4">
         <v>1.16523427811731e-06</v>
       </c>
-      <c r="D16" s="4">
+      <c r="Y16" s="4">
         <v>1.7563856964467709e-07</v>
       </c>
-      <c r="E16" s="4">
+      <c r="Z16" s="4">
         <v>0.99990411434852822</v>
       </c>
-      <c r="F16" s="4">
+      <c r="AA16" s="4">
         <v>6.6350656886910513e-07</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4">
+      <c r="A17" s="1">
+        <v>0</v>
+      </c>
+      <c r="B17" s="1">
+        <v>1</v>
+      </c>
+      <c r="C17" s="1">
+        <v>0</v>
+      </c>
+      <c r="D17" s="1">
+        <v>0</v>
+      </c>
+      <c r="E17" s="1">
+        <v>1</v>
+      </c>
+      <c r="F17" s="1">
+        <v>0</v>
+      </c>
+      <c r="H17" s="1">
+        <v>0</v>
+      </c>
+      <c r="I17" s="1">
+        <v>1</v>
+      </c>
+      <c r="J17" s="1">
+        <v>0</v>
+      </c>
+      <c r="K17" s="1">
+        <v>0</v>
+      </c>
+      <c r="L17" s="1">
+        <v>1</v>
+      </c>
+      <c r="M17" s="1">
+        <v>0</v>
+      </c>
+      <c r="O17" s="1">
+        <f>A6</f>
+        <v>0</v>
+      </c>
+      <c r="P17" s="1">
+        <f>B6</f>
+        <v>1</v>
+      </c>
+      <c r="Q17" s="1">
+        <f>C6</f>
+        <v>0</v>
+      </c>
+      <c r="R17" s="1">
+        <f>D6</f>
+        <v>0</v>
+      </c>
+      <c r="S17" s="1">
+        <f>E6</f>
+        <v>1</v>
+      </c>
+      <c r="T17" s="1">
+        <f>F6</f>
+        <v>0</v>
+      </c>
+      <c r="V17" s="4">
         <v>2.5057586375407954e-07</v>
       </c>
-      <c r="B17" s="4">
+      <c r="W17" s="4">
         <v>0.99861392117641312</v>
       </c>
-      <c r="C17" s="4">
+      <c r="X17" s="4">
         <v>7.112617049975062e-07</v>
       </c>
-      <c r="D17" s="4">
+      <c r="Y17" s="4">
         <v>1.082643862479697e-07</v>
       </c>
-      <c r="E17" s="4">
+      <c r="Z17" s="4">
         <v>0.99997855377413525</v>
       </c>
-      <c r="F17" s="4">
+      <c r="AA17" s="4">
         <v>1.3458300196942424e-06</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4">
+      <c r="A18" s="1">
+        <v>0</v>
+      </c>
+      <c r="B18" s="1">
+        <v>0</v>
+      </c>
+      <c r="C18" s="1">
+        <v>1</v>
+      </c>
+      <c r="D18" s="1">
+        <v>1</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0</v>
+      </c>
+      <c r="F18" s="1">
+        <v>0</v>
+      </c>
+      <c r="H18" s="1">
+        <v>0</v>
+      </c>
+      <c r="I18" s="1">
+        <v>0</v>
+      </c>
+      <c r="J18" s="1">
+        <v>1</v>
+      </c>
+      <c r="K18" s="1">
+        <v>1</v>
+      </c>
+      <c r="L18" s="1">
+        <v>0</v>
+      </c>
+      <c r="M18" s="1">
+        <v>0</v>
+      </c>
+      <c r="O18" s="1">
+        <f>A7</f>
+        <v>0</v>
+      </c>
+      <c r="P18" s="1">
+        <f>B7</f>
+        <v>0</v>
+      </c>
+      <c r="Q18" s="1">
+        <f>C7</f>
+        <v>1</v>
+      </c>
+      <c r="R18" s="1">
+        <f>D7</f>
+        <v>1</v>
+      </c>
+      <c r="S18" s="1">
+        <f>E7</f>
+        <v>0</v>
+      </c>
+      <c r="T18" s="1">
+        <f>F7</f>
+        <v>0</v>
+      </c>
+      <c r="V18" s="4">
         <v>4.1753757848600836e-07</v>
       </c>
-      <c r="B18" s="4">
+      <c r="W18" s="4">
         <v>0.00014785071390493041</v>
       </c>
-      <c r="C18" s="4">
+      <c r="X18" s="4">
         <v>0.99999995015981691</v>
       </c>
-      <c r="D18" s="4">
+      <c r="Y18" s="4">
         <v>0.99999996490507714</v>
       </c>
-      <c r="E18" s="4">
+      <c r="Z18" s="4">
         <v>5.0986733618889124e-05</v>
       </c>
-      <c r="F18" s="4">
+      <c r="AA18" s="4">
         <v>7.0171338710906942e-07</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4">
+      <c r="A19" s="1">
+        <v>0</v>
+      </c>
+      <c r="B19" s="1">
+        <v>0</v>
+      </c>
+      <c r="C19" s="1">
+        <v>0</v>
+      </c>
+      <c r="D19" s="1">
+        <v>0</v>
+      </c>
+      <c r="E19" s="1">
+        <v>0</v>
+      </c>
+      <c r="F19" s="1">
+        <v>0</v>
+      </c>
+      <c r="H19" s="1">
+        <v>0</v>
+      </c>
+      <c r="I19" s="1">
+        <v>0</v>
+      </c>
+      <c r="J19" s="1">
+        <v>0</v>
+      </c>
+      <c r="K19" s="1">
+        <v>0</v>
+      </c>
+      <c r="L19" s="1">
+        <v>0</v>
+      </c>
+      <c r="M19" s="1">
+        <v>0</v>
+      </c>
+      <c r="O19" s="1">
+        <f>A8</f>
+        <v>0</v>
+      </c>
+      <c r="P19" s="1">
+        <f>B8</f>
+        <v>0</v>
+      </c>
+      <c r="Q19" s="1">
+        <f>C8</f>
+        <v>0</v>
+      </c>
+      <c r="R19" s="1">
+        <f>D8</f>
+        <v>0</v>
+      </c>
+      <c r="S19" s="1">
+        <f>E8</f>
+        <v>0</v>
+      </c>
+      <c r="T19" s="1">
+        <f>F8</f>
+        <v>0</v>
+      </c>
+      <c r="V19" s="4">
         <v>4.7805073638182365e-07</v>
       </c>
-      <c r="B19" s="4">
+      <c r="W19" s="4">
         <v>1.1557971492492163e-06</v>
       </c>
-      <c r="C19" s="4">
+      <c r="X19" s="4">
         <v>1.8407007264340937e-06</v>
       </c>
-      <c r="D19" s="4">
+      <c r="Y19" s="4">
         <v>6.6762146176396315e-07</v>
       </c>
-      <c r="E19" s="4">
+      <c r="Z19" s="4">
         <v>1.0769366468967413e-06</v>
       </c>
-      <c r="F19" s="4">
+      <c r="AA19" s="4">
         <v>6.2545489270617427e-07</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:F8 H1:BC1">
+  <conditionalFormatting sqref="A1:F8 H1:BC1 A12:F19 H12:M19 O12:T19">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThanOrEqual">
       <formula>0.5</formula>
     </cfRule>
@@ -3080,7 +5555,7 @@
       <formula>0.5</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A12:F19">
+  <conditionalFormatting sqref="V12:AA19">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="0"/>

</xml_diff>